<commit_message>
Username and password in user dictionary updated
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,6 +40,12 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
+    <t xml:space="preserve">MID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TID</t>
+  </si>
+  <si>
     <t xml:space="preserve">Auto_Portal_001</t>
   </si>
   <si>
@@ -52,55 +58,28 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_Portal_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Random</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_001_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Merchant_001</t>
+    <t xml:space="preserve">Auto_007_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_Merchant_007</t>
   </si>
   <si>
     <t xml:space="preserve">Admin</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_001_002</t>
+    <t xml:space="preserve">Auto_007_002</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_002_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Merchant_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_002_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_003_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Merchant_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_003_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Portal_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_004_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Merchant_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_004_002</t>
+    <t xml:space="preserve">Auto_008_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_Merchant_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_008_002</t>
   </si>
 </sst>
 </file>
@@ -110,7 +89,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -138,11 +117,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -213,7 +187,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -294,8 +268,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.77"/>
@@ -322,227 +296,122 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>2222220100</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>2222220100</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>3333330701</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>2222220200</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="E3" s="2" t="n">
-        <v>2222220200</v>
+        <v>3333330701</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>9</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3333330101</v>
+        <v>3333330702</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3333330101</v>
+        <v>3333330702</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3333330102</v>
+        <v>3333330801</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>3333330102</v>
+        <v>3333330801</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>16</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3333330201</v>
+        <v>3333330802</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>3333330201</v>
+        <v>3333330802</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>3333330202</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>3333330202</v>
-      </c>
-      <c r="F7" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>3333330301</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>3333330301</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>3333330302</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>3333330302</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>2222220300</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>2222220300</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>3333330401</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>3333330401</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>3333330402</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>3333330402</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
DB updated for merchant creation and resource assigner
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t xml:space="preserve">AutomationSuperUser1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AutomationSuperUser2</t>
   </si>
 </sst>
 </file>
@@ -180,17 +183,13 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -283,7 +282,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -311,170 +310,182 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>8548594594</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="n">
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>8548594594</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>8548594595</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
         <v>8548594595</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>8548594590</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>8548594590</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>8548594999</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>8548594999</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>8548555446</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="3" t="n">
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>8548555446</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>8758787876</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="3" t="n">
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>8758787876</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="2" t="n">
         <v>8758787889</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="3" t="n">
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>8758787889</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
+    <row r="9" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>8758787890</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>8758787890</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="4"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="4"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Merchant creation and resource assigner completed
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="25">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -76,7 +76,7 @@
     <t xml:space="preserve">AUTOTESTMERCHANT5</t>
   </si>
   <si>
-    <t xml:space="preserve">AutomationSuperUser</t>
+    <t xml:space="preserve">SuperUserOne</t>
   </si>
   <si>
     <t xml:space="preserve">EZETAP</t>
@@ -85,10 +85,16 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">AutomationSuperUser1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AutomationSuperUser2</t>
+    <t xml:space="preserve">SuperUserTwo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperUserThree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperUserFour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperUserFive</t>
   </si>
 </sst>
 </file>
@@ -183,13 +189,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -282,7 +292,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -310,182 +320,206 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>8548594594</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>8548594594</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>8548594595</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>8548594595</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>8548594590</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>8548594590</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>8548594999</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>8548594999</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>8548555446</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
+      <c r="D6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>8548555446</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="3" t="n">
         <v>8758787876</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
+      <c r="D7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>8758787876</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>8758787889</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>8758787889</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="C8" s="3" t="n">
+        <v>8758787877</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>8758787877</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>8758787890</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>8758787890</v>
-      </c>
-      <c r="F9" s="3" t="s">
+      <c r="C9" s="3" t="n">
+        <v>8758787878</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>8758787878</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="3"/>
+      <c r="A10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>8758787879</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>8758787879</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
+      <c r="A11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>8758787870</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>8758787870</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
removed unnessary enteries of merchant creation
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,10 +40,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">automation_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOMATIONTESTMERCHANT</t>
+    <t xml:space="preserve">auto_user_test_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_Merchant_test_001</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -52,37 +52,19 @@
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">automation_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">automation_3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTO_TEST_MERCHANT_4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automation_5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT5</t>
+    <t xml:space="preserve">auto_user_test_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperUserTest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal</t>
   </si>
   <si>
     <t xml:space="preserve">SuperUserOne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
   </si>
   <si>
     <t xml:space="preserve">SuperUserTwo</t>
@@ -189,7 +171,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -198,19 +180,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -291,8 +265,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -324,201 +298,160 @@
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>8548594594</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>8548594594</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="C2" s="2" t="n">
+        <v>6666660801</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>6666660801</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>6666660803</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>6666660803</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>8548594595</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>8548594595</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>8548594590</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>8548594590</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>6666660802</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>6666660802</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>8548594999</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>8548594999</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>9</v>
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>8758787876</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>8758787876</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>8758787877</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>8758787877</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>8758787878</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>8758787878</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>8548555446</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>8548555446</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="B8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>8758787879</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>8758787879</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="3" t="n">
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="2" t="n">
         <v>8758787870</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="3" t="n">
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>8758787870</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>20</v>
+      <c r="F9" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
all test cases updated with the new finally block and added revert part before pre condition setup
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,43 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">auto_user_test_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Merchant_test_001</t>
+    <t xml:space="preserve">AVI-EULA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
   </si>
   <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
+  </si>
+  <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">auto_user_test_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserTest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserOne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserTwo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserThree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserFour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserFive</t>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -171,13 +171,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -266,7 +270,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,19 +302,19 @@
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>6666660801</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>6666660801</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="C2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -318,141 +322,117 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>6666660803</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>6666660803</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>6666660802</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>6666660802</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>13</v>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>8758787870</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>8758787870</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
changes to all the scripts
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,18 +40,24 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
+    <t xml:space="preserve">Test automation c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test automation b</t>
   </si>
   <si>
     <t xml:space="preserve">AUTOTESTMERCHANT7</t>
   </si>
   <si>
-    <t xml:space="preserve">A123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
     <t xml:space="preserve">AUTO TESTMERCHANT</t>
   </si>
   <si>
@@ -67,7 +73,10 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve"> Test automation b</t>
+    <t xml:space="preserve">Test auto sup acc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VineethB</t>
   </si>
 </sst>
 </file>
@@ -256,8 +265,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -293,19 +302,19 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5555554321</v>
+        <v>5555432100</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5555554321</v>
+        <v>5555432100</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -313,56 +322,96 @@
         <v>11</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5555543210</v>
+        <v>5555554321</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5555543210</v>
+        <v>5555554321</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>8891960880</v>
+        <v>5555543210</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>8891960880</v>
+        <v>5555543210</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="C5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>9731653475</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>9731653475</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>14</v>
+      <c r="F6" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>9731545096</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>9731545096</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added APB test cases
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,43 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">auto_user_test_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_Merchant_test_001</t>
+    <t xml:space="preserve">AVI-EULA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
   </si>
   <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
+  </si>
+  <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">auto_user_test_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserTest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserOne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserTwo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserThree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserFour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperUserFive</t>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -171,13 +171,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -266,7 +270,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,19 +302,19 @@
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>6666660801</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>6666660801</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="C2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -318,141 +322,117 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>6666660803</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>6666660803</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>6666660802</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>6666660802</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>8758787877</v>
+        <v>6789876556</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>13</v>
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>8758787878</v>
+        <v>6789343487</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>13</v>
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>8758787870</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>8758787870</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
adding bqrv4 axis cases and changed bqr cases
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -40,43 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AVI-EULA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap</t>
+    <t xml:space="preserve">AUTO TESTMERCHANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT6</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
   </si>
   <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
+  </si>
+  <si>
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
+    <t xml:space="preserve">Test auto sup acc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VineethB</t>
   </si>
 </sst>
 </file>
@@ -171,17 +171,13 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -269,8 +265,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,23 +294,23 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="C2" s="2" t="n">
+        <v>5555543210</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5555543210</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -322,117 +318,101 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5555554321</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5555554321</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5555432100</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5555432100</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F5" s="4" t="s">
         <v>14</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="n">
+        <v>9731653475</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9731653475</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
         <v>18</v>
       </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="C7" s="2" t="n">
-        <v>6789343487</v>
+        <v>9731545096</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
+        <v>9731545096</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added teardown setup method.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,43 +40,40 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AUTO TESTMERCHANT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT6</t>
+    <t xml:space="preserve">Sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANDEEPTEST_8144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q121212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ChethanCP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TESTCHETHAN_3087</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandeepkumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperUserFive</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automation b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automation c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automation a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test auto sup acc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VineethB</t>
   </si>
 </sst>
 </file>
@@ -171,7 +168,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -181,6 +178,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -265,8 +278,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -301,118 +314,86 @@
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>5555543210</v>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5555543210</v>
+        <v>1232123212</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>9191917171</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="E3" s="5" t="n">
+        <v>9988989809</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>5555554321</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>5555554321</v>
-      </c>
-      <c r="F3" s="3" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>5555432100</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="E4" s="2" t="n">
-        <v>5555432100</v>
+        <v>9988987089</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="5" t="n">
+        <v>8758787870</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>8758787870</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>8891960880</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8891960880</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>9731653475</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>9731653475</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>9731545096</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>9731545096</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A6" s="4"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
HDFC TID Dependent test cases
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -40,43 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Test automation c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
+    <t xml:space="preserve">AVI-EULA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
   </si>
   <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
+  </si>
+  <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">Test automation b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTO TESTMERCHANT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automation a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test auto sup acc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VineethB</t>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -171,13 +171,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -265,8 +269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,19 +302,19 @@
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>5555432100</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>5555432100</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="C2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -318,101 +322,117 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>5555554321</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>5555554321</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>5555543210</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>5555543210</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>8891960880</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8891960880</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>9731653475</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>9731653475</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="C7" s="2" t="n">
-        <v>9731545096</v>
+        <v>6789343487</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>9731545096</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>16</v>
-      </c>
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added new test cases for callback and refund scenarios
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,43 +40,46 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AVI-EULA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A123456</t>
+    <t xml:space="preserve">Sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANDEEPTEST_8144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q121212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remotepay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MURFY12_30802597</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JyTMsFZlfn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROMODEV_4516605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q12121212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandeepkumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
   </si>
   <si>
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
+    <t xml:space="preserve">Sandeepkumarrajak</t>
   </si>
 </sst>
 </file>
@@ -171,7 +174,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -180,16 +183,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -269,8 +276,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,141 +305,105 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
+      <c r="E2" s="2" t="n">
+        <v>1232123212</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>6360953784</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="F3" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>7736923648</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>7736923648</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F4" s="4" t="s">
+      <c r="E5" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>9880132901</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="E6" s="4" t="n">
+        <v>9880132901</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added upi cases of APB, AXIS_DIRECT, HDFC Tid_Dep and BQRV4_UPI cases of KOtak_Atos PGs
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,46 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Sandeep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SANDEEPTEST_8144</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sandeep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q121212</t>
+    <t xml:space="preserve">AVI-EULA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">Remotepay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MURFY12_30802597</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JyTMsFZlfn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROMODEV_4516605</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q12121212</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandeepkumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandeepkumarrajak</t>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -174,7 +171,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -183,20 +180,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -276,8 +269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -305,105 +298,141 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>1232123212</v>
-      </c>
-      <c r="F2" s="3" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>6360953784</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>7736923648</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="5" t="n">
-        <v>7736923648</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>9988987089</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>9988987089</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>9880132901</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>9880132901</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="C7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
tid dep cases update
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -40,43 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AVI-EULA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap</t>
+    <t xml:space="preserve">AUTO TESTMERCHANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT6</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
   </si>
   <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
+  </si>
+  <si>
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
+    <t xml:space="preserve">Test auto sup acc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VineethB</t>
   </si>
 </sst>
 </file>
@@ -171,17 +171,13 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -269,8 +265,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,23 +294,23 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="C2" s="2" t="n">
+        <v>5555543210</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5555543210</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -322,117 +318,101 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5555554321</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5555554321</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5555432100</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5555432100</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F5" s="4" t="s">
         <v>14</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="n">
+        <v>9731653475</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9731653475</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
         <v>18</v>
       </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="C7" s="2" t="n">
-        <v>6789343487</v>
+        <v>9731545096</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
+        <v>9731545096</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
fixed issues after running in jenkins and added 5 test cases for Axis Direct.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,31 +40,37 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AUTO TESTMERCHANT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A123456</t>
+    <t xml:space="preserve">Sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANDEEPTEST_8144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q121212</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">Test automation b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automation c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test automation a</t>
+    <t xml:space="preserve">JyTMsFZlfn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROMODEV_4516605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q12121212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remotepay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MURFY12_30802597</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandeepkumar</t>
   </si>
   <si>
     <t xml:space="preserve">EZETAP</t>
@@ -73,10 +79,10 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Test auto sup acc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VineethB</t>
+    <t xml:space="preserve">Sandeepkumarrajak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sandeeptest</t>
   </si>
 </sst>
 </file>
@@ -171,7 +177,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -181,11 +187,19 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -266,7 +280,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -301,123 +315,123 @@
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>5555543210</v>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5555543210</v>
+        <v>1232123212</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>7736923648</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>7736923648</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="E4" s="5" t="n">
+        <v>6360953784</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>5555554321</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>5555554321</v>
-      </c>
-      <c r="F3" s="3" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>5555432100</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>5555432100</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E5" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>9880132901</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>8891960880</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8891960880</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="E6" s="4" t="n">
+        <v>9880132901</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>9731653475</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>9731653475</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="C7" s="0" t="n">
+        <v>9775822323</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>9775822323</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>9731545096</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>9731545096</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
added KOTAK_ATOS BQRV4_BQR cases
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,49 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Sandeep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SANDEEPTEST_8144</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sandeep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q121212</t>
+    <t xml:space="preserve">AVI-EULA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">JyTMsFZlfn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROMODEV_4516605</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q12121212</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remotepay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MURFY12_30802597</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandeepkumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EZETAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandeepkumarrajak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sandeeptest</t>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -177,7 +171,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -186,20 +180,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -279,8 +269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="12.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -308,130 +298,146 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>1232123212</v>
-      </c>
-      <c r="F2" s="3" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="5" t="n">
-        <v>7736923648</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="5" t="n">
-        <v>7736923648</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>6360953784</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>9988987089</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>9988987089</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>9880132901</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>9880132901</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="0" t="n">
-        <v>9775822323</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="0" t="n">
-        <v>9775822323</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="C7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
added new test cases for Axis direct and fixed netbanking issues.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,43 +40,49 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AVI-EULA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A123456</t>
+    <t xml:space="preserve">Sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANDEEPTEST_8144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sandeep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q121212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JyTMsFZlfn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROMODEV_4516605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q12121212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remotepay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MURFY12_30802597</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandeepkumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
   </si>
   <si>
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
+    <t xml:space="preserve">Sandeepkumarrajak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sandeeptest</t>
   </si>
 </sst>
 </file>
@@ -171,7 +177,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -180,16 +186,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -269,8 +279,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="12.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,146 +308,130 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="E2" s="2" t="n">
+        <v>1232123212</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="F3" s="4" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>7736923648</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>7736923648</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F4" s="4" t="s">
+      <c r="E4" s="5" t="n">
+        <v>6360953784</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
+      <c r="E5" s="2" t="n">
+        <v>9988987089</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>9880132901</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>9880132901</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="0" t="n">
+        <v>9775822323</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>9775822323</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
Merchant creation enhancement completed.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="AcquisitionDetails" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -41,10 +42,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch15</t>
+    <t xml:space="preserve">Auto_test_user13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch13</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -53,10 +54,10 @@
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch16</t>
+    <t xml:space="preserve">Auto_test_user14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch14</t>
   </si>
   <si>
     <t xml:space="preserve">Acquirer Code</t>
@@ -71,34 +72,67 @@
     <t xml:space="preserve">HSM Name</t>
   </si>
   <si>
+    <t xml:space="preserve">HDFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AXIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVI-EULA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICICI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATOS_TLE</t>
+  </si>
+  <si>
     <t xml:space="preserve">KOTAK</t>
   </si>
   <si>
     <t xml:space="preserve">KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICICI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AXIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATOS_TLE</t>
   </si>
   <si>
     <t xml:space="preserve">AIRP</t>
@@ -114,7 +148,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -142,6 +176,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -199,7 +238,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -216,11 +255,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -302,7 +337,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -330,7 +365,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -338,19 +373,19 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>9410178815</v>
+        <v>9300178815</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9410178815</v>
+        <v>9300178815</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -358,13 +393,13 @@
         <v>11</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>9410178816</v>
+        <v>9300178816</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9410178816</v>
+        <v>9300178816</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>9</v>
@@ -386,145 +421,298 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="0" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>1</v>
+      <c r="B2" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="2" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="n">
+        <v>9660867345</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>9660867344</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="B12" s="0" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="C12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="B15" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
+      <c r="B18" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
merchant creation file cleaned up
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -10,7 +10,6 @@
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="AcquisitionDetails" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -79,66 +78,6 @@
   </si>
   <si>
     <t xml:space="preserve">AXIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVI-EULA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICICI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATOS_TLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KOTAK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KOTAK_ATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIRP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APB</t>
   </si>
 </sst>
 </file>
@@ -148,7 +87,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -176,11 +115,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -255,7 +189,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -337,7 +271,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -422,13 +356,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.88"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -476,243 +410,6 @@
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="2" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="2" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>17</v>
-      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Terminal details db udpate completed
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="AcquisitionDetails" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -41,10 +42,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch18</t>
+    <t xml:space="preserve">Auto_test_user24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch24</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -296,7 +297,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -332,13 +333,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>9511188815</v>
+        <v>8921188815</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9511188815</v>
+        <v>8921188815</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -369,7 +370,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -434,79 +435,98 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Merchant name added to terminal_details table
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -297,7 +297,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -370,7 +370,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -456,7 +456,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">

</xml_diff>

<commit_message>
added new cases of fdc and bqrv4_upi for axis_direct
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Manasa</t>
+    <t xml:space="preserve">AVI-EULA</t>
   </si>
   <si>
     <t xml:space="preserve">Ezetap</t>
@@ -52,13 +52,31 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">anika</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CNPAUTOMATIONPHASEI</t>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -251,8 +269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -280,7 +298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -288,13 +306,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>7204644212</v>
+        <v>9660867345</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>7204644212</v>
+        <v>9660867345</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>9</v>
@@ -304,29 +322,117 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>7207207209</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>7207207209</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="4"/>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Merchant config initial commit
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,12 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="AcquisitionDetails" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="41">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -66,15 +65,48 @@
     <t xml:space="preserve">HSM Name</t>
   </si>
   <si>
+    <t xml:space="preserve">Bank Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQR Bank Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPI(psp) Bank Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BQR Terminal Dependant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPI Terminal Dependant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key for UPI</t>
+  </si>
+  <si>
     <t xml:space="preserve">HDFC</t>
   </si>
   <si>
     <t xml:space="preserve">NONE</t>
   </si>
   <si>
+    <t xml:space="preserve">True</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57c3f7c3b0d8dc0be189ec63f68fce42</t>
+  </si>
+  <si>
     <t xml:space="preserve">AXIS</t>
   </si>
   <si>
+    <t xml:space="preserve">AXIS_DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">False</t>
+  </si>
+  <si>
     <t xml:space="preserve">YES</t>
   </si>
   <si>
@@ -87,27 +119,40 @@
     <t xml:space="preserve">FDC</t>
   </si>
   <si>
+    <t xml:space="preserve">FDC_ICICI</t>
+  </si>
+  <si>
     <t xml:space="preserve">ATOS_TLE</t>
   </si>
   <si>
+    <t xml:space="preserve">AXIS_TLE</t>
+  </si>
+  <si>
     <t xml:space="preserve">KOTAK</t>
   </si>
   <si>
     <t xml:space="preserve">KOTAK_ATOS</t>
   </si>
   <si>
+    <t xml:space="preserve">KOTAK_WL</t>
+  </si>
+  <si>
     <t xml:space="preserve">AIRP</t>
   </si>
   <si>
     <t xml:space="preserve">APB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal Dependant</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -194,7 +239,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -212,6 +257,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -297,7 +350,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -369,14 +422,19 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AA16"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="33.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="17.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -392,143 +450,297 @@
       <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="E1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
+      <c r="E4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA8" s="0" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA9" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J16" s="7"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I9" type="list">
+      <formula1>AcquisitionDetails!$AA$9:$AA$9</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
BQI setting thru API in progress
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="44">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -41,10 +41,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch24</t>
+    <t xml:space="preserve">Auto_test_user25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch25</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -53,6 +53,12 @@
     <t xml:space="preserve">App</t>
   </si>
   <si>
+    <t xml:space="preserve">Auto_test_user26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch26</t>
+  </si>
+  <si>
     <t xml:space="preserve">Acquirer Code</t>
   </si>
   <si>
@@ -83,6 +89,9 @@
     <t xml:space="preserve">Key for UPI</t>
   </si>
   <si>
+    <t xml:space="preserve">virtual MID Required</t>
+  </si>
+  <si>
     <t xml:space="preserve">HDFC</t>
   </si>
   <si>
@@ -95,6 +104,9 @@
     <t xml:space="preserve">57c3f7c3b0d8dc0be189ec63f68fce42</t>
   </si>
   <si>
+    <t xml:space="preserve">False</t>
+  </si>
+  <si>
     <t xml:space="preserve">AXIS</t>
   </si>
   <si>
@@ -102,9 +114,6 @@
   </si>
   <si>
     <t xml:space="preserve">N/A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">False</t>
   </si>
   <si>
     <t xml:space="preserve">YES</t>
@@ -350,7 +359,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -386,25 +395,37 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8921188815</v>
+        <v>8921188816</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8921188815</v>
+        <v>8921188816</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>8921188916</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>8921188916</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -423,7 +444,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -431,97 +452,104 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="33.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="33.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="17.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>27</v>
@@ -530,30 +558,33 @@
         <v>27</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>27</v>
@@ -562,62 +593,68 @@
         <v>27</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>26</v>
+      <c r="K5" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>27</v>
@@ -626,30 +663,33 @@
         <v>27</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>27</v>
@@ -658,30 +698,33 @@
         <v>27</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>27</v>
@@ -690,33 +733,36 @@
         <v>27</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="AA8" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>27</v>
@@ -725,10 +771,13 @@
         <v>27</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="AA9" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -736,7 +785,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I9" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I9 K2:K9" type="list">
       <formula1>AcquisitionDetails!$AA$9:$AA$9</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
UPI settings implementation completed.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
@@ -41,10 +41,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch27</t>
+    <t xml:space="preserve">Auto_test_user28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch28</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -353,7 +353,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.0546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -389,13 +389,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8921188817</v>
+        <v>8921188818</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8921188817</v>
+        <v>8921188818</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -426,7 +426,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>

</xml_diff>

<commit_message>
UPI setting through db completed.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -41,10 +41,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch28</t>
+    <t xml:space="preserve">Auto_test_user29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch29</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -353,7 +353,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -389,13 +389,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8921188818</v>
+        <v>8921188819</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8921188818</v>
+        <v>8921188819</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -426,7 +426,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -528,7 +528,7 @@
         <v>27</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>26</v>
@@ -703,7 +703,7 @@
         <v>40</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
cnp setting implementation completed
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,11 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="AcquisitionDetails" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="RemotepaySettings" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="PgDetails" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="90">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -41,10 +43,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch29</t>
+    <t xml:space="preserve">Auto_test_user31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch31</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -147,6 +149,150 @@
   </si>
   <si>
     <t xml:space="preserve">Terminal Dependant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Component</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LockId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EntityId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inheritable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cnpTxnTimeoutDuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_binary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximumPayAttemptsAllowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maxUpiAttemptInCNP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remotePayExpTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rmpayBumpCount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rmpayBumpTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upiCollectEnableOnAndroidDevice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upiCollectEnableOnNonAndroidDevices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLIENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upiEnabledInCNP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Api Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Api Key2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secret2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Api Key3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secret3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lock Id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hash Algo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mle Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nb Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nb Selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cnp Cardpay Enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account Label Id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transaction Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CYBERSOURCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DV+y0pRK1jhkpBipZ+YtM06XqQGOi1SDwsmOY/K4wqo=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8bf3bb8f-eb7c-45d2-b227-bf779907d017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezetap_2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INACTIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPSL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2989436385NXGVOA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4053377546CSKYIV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T297100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIRST_amount_0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">470|TPSL Bank::</t>
   </si>
 </sst>
 </file>
@@ -157,7 +303,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -185,6 +331,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -242,7 +393,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -272,6 +423,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -353,7 +512,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -389,13 +548,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8921188819</v>
+        <v>8921188821</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8921188819</v>
+        <v>8921188821</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -426,7 +585,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -525,13 +684,13 @@
         <v>22</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>26</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>25</v>
@@ -601,7 +760,7 @@
         <v>33</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>25</v>
@@ -780,4 +939,428 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.58"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>10786</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="49.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="20.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="15.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="18.77"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>120000000008131</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>120000000008131</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>120000000008131</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
CNP cases and offline refund ATOS_TLE
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,7 +41,7 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AVI-EULA</t>
+    <t xml:space="preserve">Manasa</t>
   </si>
   <si>
     <t xml:space="preserve">Ezetap</t>
@@ -52,31 +53,13 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
+    <t xml:space="preserve">anika</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNPAUTOMATIONPHASEI</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -269,8 +252,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,7 +281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -306,133 +289,69 @@
         <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9660867345</v>
+        <v>7204644212</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>9660867345</v>
+        <v>7204644212</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9660867344</v>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>7207207209</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="n">
-        <v>9660867344</v>
+      <c r="E3" s="2" t="n">
+        <v>7207207209</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -443,4 +362,43 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="n">
+        <v>7207207209</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="n">
+        <v>7207207209</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added new cases of bqrv4_upi of axis_direct
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -9,7 +9,6 @@
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -41,7 +40,7 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Manasa</t>
+    <t xml:space="preserve">AVI-EULA</t>
   </si>
   <si>
     <t xml:space="preserve">Ezetap</t>
@@ -53,13 +52,31 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">anika</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CNPAUTOMATIONPHASEI</t>
+    <t xml:space="preserve">Avin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avinash-one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI_7</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinash-hdfc-two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTESTUPI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avinashthree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVINASHTEST2_355</t>
   </si>
 </sst>
 </file>
@@ -252,8 +269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -281,7 +298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -289,69 +306,133 @@
         <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>7204644212</v>
+        <v>9660867345</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>7204644212</v>
+        <v>9660867345</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>9660867344</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>7207207209</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>7207207209</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9660867300</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7897485874</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="4"/>
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6789876556</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="4"/>
+      <c r="A7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>6789343487</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -362,43 +443,4 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="2" t="n">
-        <v>7207207209</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="2" t="n">
-        <v>7207207209</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Merchant configuration progress check-in 1
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
@@ -43,10 +43,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch32</t>
+    <t xml:space="preserve">Auto_test_user41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch41</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -515,7 +515,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -551,13 +551,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8921188822</v>
+        <v>8922188831</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8921188822</v>
+        <v>8922188831</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -588,7 +588,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -763,7 +763,7 @@
         <v>27</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>28</v>
@@ -804,7 +804,7 @@
         <v>27</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>28</v>
@@ -845,7 +845,7 @@
         <v>27</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>28</v>
@@ -886,7 +886,7 @@
         <v>27</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>28</v>
@@ -971,7 +971,7 @@
         <v>25</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>28</v>
@@ -1006,7 +1006,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1258,7 +1258,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>

</xml_diff>

<commit_message>
Merchant configuration for upi completed.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="96">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -43,10 +43,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch41</t>
+    <t xml:space="preserve">Auto_test_user45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch45</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">UPI Terminal Dependant</t>
   </si>
   <si>
-    <t xml:space="preserve">Key for UPI</t>
+    <t xml:space="preserve">App Key for UPI</t>
   </si>
   <si>
     <t xml:space="preserve">virtual MID Required</t>
@@ -94,6 +94,9 @@
     <t xml:space="preserve">UPI settings required</t>
   </si>
   <si>
+    <t xml:space="preserve">Enc Key for UPI</t>
+  </si>
+  <si>
     <t xml:space="preserve">HDFC</t>
   </si>
   <si>
@@ -112,15 +115,15 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
+    <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
     <t xml:space="preserve">AXIS</t>
   </si>
   <si>
     <t xml:space="preserve">AXIS_DIRECT</t>
   </si>
   <si>
-    <t xml:space="preserve">N/A</t>
-  </si>
-  <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
@@ -160,7 +163,10 @@
     <t xml:space="preserve">APB</t>
   </si>
   <si>
-    <t xml:space="preserve">Terminal Dependant</t>
+    <t xml:space="preserve">4ba841d6-c012-4d19-ab49-2ee74366171p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7f617238-fb82-4b</t>
   </si>
   <si>
     <t xml:space="preserve">Value</t>
@@ -425,11 +431,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -515,7 +521,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -551,13 +557,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8922188831</v>
+        <v>8922188835</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8922188831</v>
+        <v>8922188835</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -587,8 +593,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AA53"/>
+  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -598,10 +604,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="33.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="38.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="19.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="17.74"/>
   </cols>
   <sheetData>
@@ -645,348 +652,379 @@
       <c r="M1" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="N1" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="M6" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="0" t="s">
-        <v>45</v>
+        <v>29</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="M9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA9" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J16" s="7"/>
+      <c r="N9" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J15" s="6"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AA52" s="7"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AA53" s="7"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I9 K2:K9" type="list">
-      <formula1>AcquisitionDetails!$AA$9:$AA$9</formula1>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K9" type="list">
+      <formula1>AcquisitionDetails!$AA$52:$AA$52</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I9" type="list">
+      <formula1>AcquisitionDetails!$AA$52:$AA$53</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1006,7 +1044,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1016,229 +1054,229 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>10786</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1258,7 +1296,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>
@@ -1275,60 +1313,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>120000000008131</v>
@@ -1340,29 +1378,29 @@
         <v>120000000008131</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3" t="n">
@@ -1371,42 +1409,42 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3" t="n">

</xml_diff>

<commit_message>
UPI and BQR implementation completed.
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
@@ -43,10 +43,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch45</t>
+    <t xml:space="preserve">Auto_test_user46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch46</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -521,7 +521,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.2890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.31640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -557,13 +557,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8922188835</v>
+        <v>8922188836</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8922188835</v>
+        <v>8922188836</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -594,7 +594,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -1044,7 +1044,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1296,7 +1296,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>

</xml_diff>

<commit_message>
CNP settings issue fixed
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -43,10 +43,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch46</t>
+    <t xml:space="preserve">Auto_test_user49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch49</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -521,7 +521,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.31640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -557,13 +557,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8922188836</v>
+        <v>8922188839</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8922188836</v>
+        <v>8922188839</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -594,7 +594,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -1044,7 +1044,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1296,7 +1296,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>

</xml_diff>

<commit_message>
org settings implementation complete
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -12,6 +12,7 @@
     <sheet name="AcquisitionDetails" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="RemotepaySettings" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="PgDetails" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="OrgSettings" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="105">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -43,10 +44,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch49</t>
+    <t xml:space="preserve">Auto_test_user50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch50</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -311,6 +312,33 @@
   </si>
   <si>
     <t xml:space="preserve">470|TPSL Bank::</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setting Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setting Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upiEnabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qrCodesEnabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BHARAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remotePaymentEnabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ctlsEnabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refundEnabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">onlineRefundEnabled</t>
   </si>
 </sst>
 </file>
@@ -406,7 +434,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -441,6 +469,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -521,7 +553,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -557,13 +589,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8922188839</v>
+        <v>8922188840</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8922188839</v>
+        <v>8922188840</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -594,7 +626,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -1044,7 +1076,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1296,7 +1328,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>
@@ -1460,4 +1492,152 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.74"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="9"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="9"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="9"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="9"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="9"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="9"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="9"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="9"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="9"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="9"/>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="9"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="9"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Commit before branch refresh
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -44,10 +44,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch57</t>
+    <t xml:space="preserve">Auto_test_user58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch58</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -556,7 +556,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -592,13 +592,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8922188847</v>
+        <v>8922188848</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8922188847</v>
+        <v>8922188848</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -629,7 +629,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -1079,7 +1079,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1331,7 +1331,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>
@@ -1519,7 +1519,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.74"/>

</xml_diff>

<commit_message>
Commit after branch refresh
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -44,10 +44,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto_test_user58</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto_test_merch58</t>
+    <t xml:space="preserve">Auto_test_user59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto_test_merch59</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -556,7 +556,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="12.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -592,13 +592,13 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>8922188848</v>
+        <v>8922188849</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>8922188848</v>
+        <v>8922188849</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
@@ -629,7 +629,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.45"/>
@@ -1079,7 +1079,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.59"/>
   </cols>
@@ -1331,7 +1331,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.44"/>
@@ -1519,7 +1519,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.74"/>

</xml_diff>

<commit_message>
mergin all the tcs
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -40,43 +40,43 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">AVI-EULA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap</t>
+    <t xml:space="preserve">AUTO TESTMERCHANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT6</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
   </si>
   <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTOTESTMERCHANT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test automation a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EZETAP</t>
+  </si>
+  <si>
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Avin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avinash-one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinash-hdfc-two</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTESTUPI1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avinashthree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVINASHTEST2_355</t>
+    <t xml:space="preserve">Test auto sup acc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VineethB</t>
   </si>
 </sst>
 </file>
@@ -171,17 +171,13 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -269,8 +265,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42.92"/>
@@ -298,23 +294,23 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>9660867345</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="C2" s="2" t="n">
+        <v>5555543210</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5555543210</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -322,117 +318,101 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>9660867344</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5555554321</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5555554321</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>9660867300</v>
-      </c>
-      <c r="F4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5555432100</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5555432100</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7897485874</v>
-      </c>
-      <c r="F5" s="4" t="s">
         <v>14</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>8891960880</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="n">
+        <v>9731653475</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9731653475</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>6789876556</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
         <v>18</v>
       </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="C7" s="2" t="n">
-        <v>6789343487</v>
+        <v>9731545096</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6789343487</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
+        <v>9731545096</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Merchant creation Utility changes in merchant_user_creation.xlsx and ezeauto.db and merchant_creator.py
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="130">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTIACCOUNTTESTMERCHANT1</t>
+    <t xml:space="preserve">TESTMERCHFEBONE02</t>
   </si>
   <si>
     <t xml:space="preserve">App</t>
@@ -374,6 +374,9 @@
   </si>
   <si>
     <t xml:space="preserve">defaultAccount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qrCodePaymentEnabled</t>
   </si>
   <si>
     <t xml:space="preserve">ConfigMerchant</t>
@@ -423,7 +426,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -451,6 +454,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -514,7 +522,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -537,6 +545,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -649,7 +661,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.92"/>
@@ -701,19 +713,19 @@
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9872342331</v>
+        <v>2223442331</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="n">
-        <v>9872342331</v>
-      </c>
-      <c r="F3" s="6" t="s">
+      <c r="E3" s="6" t="n">
+        <v>2223442331</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="0"/>
@@ -795,7 +807,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="15.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.84765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.45"/>
@@ -814,46 +826,46 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="8" t="s">
         <v>28</v>
       </c>
       <c r="O1" s="5" t="s">
@@ -864,46 +876,46 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="9" t="s">
         <v>37</v>
       </c>
       <c r="O2" s="5" t="s">
@@ -914,46 +926,46 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="9" t="s">
         <v>34</v>
       </c>
       <c r="O3" s="5" t="s">
@@ -964,46 +976,46 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="C4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="N4" s="9" t="s">
         <v>34</v>
       </c>
       <c r="O4" s="5" t="s">
@@ -1014,46 +1026,46 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="C5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="M5" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N5" s="8" t="s">
+      <c r="N5" s="9" t="s">
         <v>34</v>
       </c>
       <c r="O5" s="5" t="s">
@@ -1064,46 +1076,46 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="C6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="L6" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="M6" s="8" t="s">
+      <c r="M6" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="8" t="s">
+      <c r="N6" s="9" t="s">
         <v>34</v>
       </c>
       <c r="O6" s="5" t="s">
@@ -1114,46 +1126,46 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>50</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K7" s="9" t="s">
+      <c r="K7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="L7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="N7" s="9" t="s">
         <v>34</v>
       </c>
       <c r="O7" s="5" t="s">
@@ -1164,46 +1176,46 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="C8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="K8" s="9" t="s">
+      <c r="K8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L8" s="8" t="s">
+      <c r="L8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M8" s="8" t="s">
+      <c r="M8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N8" s="8" t="s">
+      <c r="N8" s="9" t="s">
         <v>56</v>
       </c>
       <c r="O8" s="5" t="s">
@@ -1214,46 +1226,46 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="N9" s="9" t="s">
         <v>34</v>
       </c>
       <c r="O9" s="5" t="s">
@@ -1265,10 +1277,10 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="AA52" s="10"/>
+      <c r="AA52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="AA53" s="10"/>
+      <c r="AA53" s="11"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1297,238 +1309,238 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="15.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D2" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="9" t="n">
         <v>10786</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1549,7 +1561,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="15.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.44"/>
@@ -1558,7 +1570,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="49.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="15.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="15.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="20.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="15.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18.77"/>
@@ -1566,151 +1578,151 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="9" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="9" t="n">
         <v>120000000008131</v>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D2" s="9" t="n">
         <v>120000000008131</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="9" t="n">
         <v>120000000008131</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8" t="s">
+      <c r="M2" s="9"/>
+      <c r="N2" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8" t="n">
+      <c r="O2" s="9"/>
+      <c r="P2" s="9" t="n">
         <v>-1</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8" t="s">
+      <c r="F3" s="9"/>
+      <c r="G3" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8" t="n">
+      <c r="H3" s="9"/>
+      <c r="I3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8" t="n">
+      <c r="O3" s="9"/>
+      <c r="P3" s="9" t="n">
         <v>-1</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="10" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1737,65 +1749,65 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="15.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1803,75 +1815,80 @@
       <c r="A8" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="10"/>
+      <c r="A9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10"/>
+      <c r="B10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="10"/>
+      <c r="B11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="10"/>
+      <c r="B12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10"/>
+      <c r="B13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10"/>
+      <c r="B14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10"/>
+      <c r="B15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10"/>
+      <c r="B16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10"/>
+      <c r="B17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="10"/>
+      <c r="B18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="10"/>
+      <c r="B19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="10"/>
+      <c r="B20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="10"/>
+      <c r="B21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="10"/>
+      <c r="B22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="10"/>
+      <c r="B23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="10"/>
+      <c r="B24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="10"/>
+      <c r="B25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="10"/>
+      <c r="B26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="10"/>
+      <c r="B27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="10"/>
+      <c r="B28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="10"/>
+      <c r="B29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="10"/>
+      <c r="B30" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1890,7 +1907,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="14.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.87"/>
@@ -1899,7 +1916,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1912,58 +1929,58 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="B2" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="13" t="n">
         <v>7207207201</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="B3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="B3" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="13" t="n">
         <v>7207207202</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="B4" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="13" t="n">
         <v>7207207203</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="B5" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="13" t="n">
         <v>7207207205</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="13" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1984,15 +2001,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.3984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="13" width="17.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="13" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="14" width="17.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="14" width="18.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2006,10 +2023,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>7383838389</v>
@@ -2019,16 +2036,16 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="B3" s="13" t="s">
+      <c r="A3" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="14" t="n">
         <v>9886592527</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="14" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added portal automation into existing scripts
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="142">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -47,31 +47,34 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">visweswara rao</t>
+    <t xml:space="preserve">Dev11_Test_Shashi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev11_TestShashi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eze@1234</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EzeSuperUserShashi11</t>
   </si>
   <si>
     <t xml:space="preserve">EZETAP</t>
   </si>
   <si>
-    <t xml:space="preserve">V1234567</t>
-  </si>
-  <si>
     <t xml:space="preserve">Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">visuPlaywright</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev11_PlaywrightTest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VisuPlaywright_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PlaywrightTest_Dev11</t>
+    <t xml:space="preserve">Dev11_Test_Shashi2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev11_TestShashi2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EzeSuperUserShashi112</t>
   </si>
   <si>
     <t xml:space="preserve">Acquirer Code</t>
@@ -460,7 +463,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -494,6 +497,13 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -572,7 +582,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -580,11 +594,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -628,7 +638,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -709,8 +719,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="17.31640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="17.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.92"/>
@@ -742,19 +752,19 @@
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>9988776612</v>
-      </c>
-      <c r="D2" s="3" t="s">
+        <v>9945377288</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>9988776612</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="5" t="n">
+        <v>9945377288</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -762,43 +772,69 @@
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>9550586898</v>
-      </c>
-      <c r="D3" s="3" t="s">
+        <v>9945377299</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="n">
-        <v>9550586898</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="5" t="n">
+        <v>9945377299</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>9416350052</v>
-      </c>
-      <c r="D4" s="0" t="s">
+      <c r="C4" s="1" t="n">
+        <v>9945377280</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="0" t="n">
-        <v>9416350052</v>
-      </c>
-      <c r="F4" s="0" t="s">
+      <c r="E4" s="5" t="n">
+        <v>9945377280</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>9945377290</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>9945377290</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="eze@1234"/>
+    <hyperlink ref="D3" r:id="rId2" display="eze@1234"/>
+    <hyperlink ref="D4" r:id="rId3" display="eze@1234"/>
+    <hyperlink ref="D5" r:id="rId4" display="eze@1234"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -815,7 +851,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="16.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.45"/>
@@ -835,504 +871,504 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>31</v>
-      </c>
       <c r="F2" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O2" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P2" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C3" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="K4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J4" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>34</v>
-      </c>
       <c r="O4" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="K5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="N5" s="9" t="s">
-        <v>34</v>
-      </c>
       <c r="O5" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="N6" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="O6" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J7" s="9" t="s">
-        <v>34</v>
-      </c>
       <c r="K7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="L7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>34</v>
-      </c>
       <c r="O7" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N8" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P8" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="P9" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="O9" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P9" s="8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="P10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="K10" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="M10" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="N10" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="O10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P10" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA10" s="3"/>
+      <c r="AA10" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1368,7 +1404,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="16.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.59"/>
   </cols>
@@ -1378,229 +1414,229 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" s="9" t="n">
         <v>8</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F2" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B4" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B6" s="9" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>75</v>
-      </c>
       <c r="C9" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>10786</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1620,7 +1656,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="16.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.44"/>
@@ -1638,63 +1674,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P1" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q1" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>120000000008131</v>
@@ -1706,83 +1742,83 @@
         <v>120000000008131</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I2" s="9" t="n">
         <v>5</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M2" s="9"/>
       <c r="N2" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O2" s="9"/>
       <c r="P2" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H3" s="9"/>
       <c r="I3" s="9" t="n">
         <v>2</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O3" s="9"/>
       <c r="P3" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="Q3" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1808,7 +1844,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="16.30078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.12890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.74"/>
@@ -1816,74 +1852,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1966,7 +2002,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="15.90234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.73046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.87"/>
@@ -1975,7 +2011,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1989,58 +2025,58 @@
     </row>
     <row r="2" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C2" s="15" t="n">
         <v>7207207201</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C3" s="15" t="n">
         <v>7207207202</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C4" s="15" t="n">
         <v>7207207203</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>7207207205</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2060,15 +2096,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="14.390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="17.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="17.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="18.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2082,30 +2118,30 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C2" s="16" t="n">
         <v>7383838389</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="A3" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="6" t="n">
         <v>9886592527</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>122</v>
+      <c r="D3" s="6" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2125,47 +2161,47 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.15625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="15.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="23.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="24.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="24.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="15.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="6" width="23.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="6" width="24.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="24.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B2" s="16" t="n">
         <v>7771111110</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>7674527291947120</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
modified BQRV4 test cases for portal validation automation with playwright
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="138">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -47,10 +47,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Dev17_Test_617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev57_PlaywrightTest_61</t>
+    <t xml:space="preserve">Dev17_Test_829</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev78_PlaywrightTest_89</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -59,22 +59,13 @@
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">EzeAutoSuperUser-961</t>
+    <t xml:space="preserve">EzeAutoSuperUser-893</t>
   </si>
   <si>
     <t xml:space="preserve">EZETAP</t>
   </si>
   <si>
     <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev17_Test_617_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev57_PlaywrightTest_61_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EzeAutoSuperUser-961_2</t>
   </si>
   <si>
     <t xml:space="preserve">Acquirer Code</t>
@@ -572,11 +563,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -705,8 +696,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="17.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="17.046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.92"/>
@@ -738,19 +729,19 @@
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>7438324729</v>
-      </c>
-      <c r="D2" s="3" t="s">
+        <v>8838383839</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>7438324729</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="5" t="n">
+        <v>8838383839</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -762,63 +753,17 @@
         <v>11</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>9274092295</v>
-      </c>
-      <c r="D3" s="3" t="s">
+        <v>7377338838</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="n">
-        <v>9274092295</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="5" t="n">
+        <v>7377338838</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>7498929333</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>7498929333</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>9243222111</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>9243222111</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G7" s="0"/>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G8" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -837,7 +782,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="16.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.45"/>
@@ -857,504 +802,504 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="O1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="9" t="s">
+      <c r="L2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="M2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="O2" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="P2" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="9" t="s">
+      <c r="L3" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="M3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="9" t="s">
+      <c r="N3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="M3" s="8" t="s">
+      <c r="P3" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="L4" s="8" t="s">
+      <c r="P4" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="M4" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N4" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="L5" s="8" t="s">
+      <c r="P5" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="M5" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N5" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H6" s="9" t="s">
+      <c r="I6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="L6" s="8" t="s">
+      <c r="P6" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="J7" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="M7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="L7" s="8" t="s">
+      <c r="P7" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="M7" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N7" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P7" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="I8" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="O8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="M8" s="8" t="s">
+      <c r="P8" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="N8" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P8" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="L9" s="8" t="s">
+      <c r="P9" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="M9" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N9" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="11" t="s">
+      <c r="I10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="O10" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="K10" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="L10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M10" s="7" t="s">
+      <c r="P10" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="N10" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P10" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="AA10" s="3"/>
+      <c r="AA10" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1390,7 +1335,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.59"/>
   </cols>
@@ -1400,229 +1345,229 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1642,7 +1587,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.44"/>
@@ -1660,63 +1605,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>120000000008131</v>
@@ -1728,83 +1673,83 @@
         <v>120000000008131</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I2" s="8" t="n">
         <v>5</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="M2" s="8"/>
       <c r="N2" s="8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="O2" s="8"/>
       <c r="P2" s="8" t="n">
         <v>-1</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>106</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="O3" s="8"/>
       <c r="P3" s="8" t="n">
         <v>-1</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1830,7 +1775,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="16.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.74"/>
@@ -1838,74 +1783,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1988,7 +1933,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="15.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.87"/>
@@ -1997,7 +1942,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2011,10 +1956,10 @@
     </row>
     <row r="2" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C2" s="14" t="n">
         <v>7207207201</v>
@@ -2025,10 +1970,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C3" s="14" t="n">
         <v>7207207202</v>
@@ -2039,10 +1984,10 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>7207207203</v>
@@ -2053,10 +1998,10 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>7207207205</v>
@@ -2082,15 +2027,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="14.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="17.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="17.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="18.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2104,10 +2049,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C2" s="15" t="n">
         <v>7383838389</v>
@@ -2117,16 +2062,16 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="4" t="n">
         <v>9886592527</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2147,47 +2092,47 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="12.19140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="15.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="23.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="24.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="24.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="15.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="23.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="24.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="24.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>134</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B2" s="15" t="n">
         <v>7771111110</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D2" s="15" t="n">
         <v>7674527291947120</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Merchant Portal Automation for CNP, RemotePay
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="141">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -47,10 +47,10 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Dev17_Test_829</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev78_PlaywrightTest_89</t>
+    <t xml:space="preserve">Dev17_Test_617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev57_PlaywrightTest_61</t>
   </si>
   <si>
     <t xml:space="preserve">A123456</t>
@@ -59,13 +59,22 @@
     <t xml:space="preserve">App</t>
   </si>
   <si>
-    <t xml:space="preserve">EzeAutoSuperUser-893</t>
+    <t xml:space="preserve">EzeAutoSuperUser-961</t>
   </si>
   <si>
     <t xml:space="preserve">EZETAP</t>
   </si>
   <si>
     <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev17_Test_617_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev57_PlaywrightTest_61_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EzeAutoSuperUser-961_2</t>
   </si>
   <si>
     <t xml:space="preserve">Acquirer Code</t>
@@ -563,11 +572,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -696,8 +705,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="17.046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="17.18359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.92"/>
@@ -729,19 +738,19 @@
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>8838383839</v>
-      </c>
-      <c r="D2" s="4" t="s">
+        <v>7438324729</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="n">
-        <v>8838383839</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="1" t="n">
+        <v>7438324729</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -753,17 +762,63 @@
         <v>11</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>7377338838</v>
-      </c>
-      <c r="D3" s="4" t="s">
+        <v>9274092295</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="n">
-        <v>7377338838</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="E3" s="3" t="n">
+        <v>9274092295</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>12</v>
       </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>7498929333</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>7498929333</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>9243222111</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>9243222111</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G7" s="0"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G8" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -782,7 +837,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="16.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.45"/>
@@ -802,504 +857,504 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P2" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G3" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" s="8" t="s">
+      <c r="P3" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P8" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="M8" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="N8" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="P8" s="7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P10" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="N10" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="P10" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="AA10" s="4"/>
+      <c r="AA10" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1335,7 +1390,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="16.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.59"/>
   </cols>
@@ -1345,229 +1400,229 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>73</v>
-      </c>
       <c r="C10" s="8" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>10786</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1587,7 +1642,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="16.35546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.44"/>
@@ -1605,63 +1660,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>120000000008131</v>
@@ -1673,83 +1728,83 @@
         <v>120000000008131</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I2" s="8" t="n">
         <v>5</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="M2" s="8"/>
       <c r="N2" s="8" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="O2" s="8"/>
       <c r="P2" s="8" t="n">
         <v>-1</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="O3" s="8"/>
       <c r="P3" s="8" t="n">
         <v>-1</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1775,7 +1830,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="16.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.74"/>
@@ -1783,74 +1838,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1933,7 +1988,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="15.6328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.76953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.87"/>
@@ -1942,7 +1997,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1956,10 +2011,10 @@
     </row>
     <row r="2" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C2" s="14" t="n">
         <v>7207207201</v>
@@ -1970,10 +2025,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C3" s="14" t="n">
         <v>7207207202</v>
@@ -1984,10 +2039,10 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>7207207203</v>
@@ -1998,10 +2053,10 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>7207207205</v>
@@ -2027,15 +2082,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="14.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="17.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="17.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="18.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2049,10 +2104,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C2" s="15" t="n">
         <v>7383838389</v>
@@ -2062,16 +2117,16 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="A3" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="3" t="n">
         <v>9886592527</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2092,47 +2147,47 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="12.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.19140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="15.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="13.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="23.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="24.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="24.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="15.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="23.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="24.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="24.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B2" s="15" t="n">
         <v>7771111110</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D2" s="15" t="n">
         <v>7674527291947120</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Testcase details file and merchant_user_creation
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="158">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -50,67 +50,73 @@
     <t xml:space="preserve">Category</t>
   </si>
   <si>
-    <t xml:space="preserve">EzeAutoSuperUser-1</t>
+    <t xml:space="preserve">Portaltanuja</t>
   </si>
   <si>
     <t xml:space="preserve">EZETAP</t>
   </si>
   <si>
+    <t xml:space="preserve">P123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P123457</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P123458</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P123459</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portal4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P123460</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARDNEWNOV_20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A123456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARDNEWNOV_21</t>
+  </si>
+  <si>
     <t xml:space="preserve">A123457</t>
   </si>
   <si>
-    <t xml:space="preserve">Portal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EzeAutoSuperUser-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EzeAutoSuperUser-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EzeAutoSuperUser-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EzeAutoSuperUser-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A123456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEV16AUTOTEST_10</t>
+    <t xml:space="preserve">CARDNEWNOV_22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A123458</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARDNEWNOV_23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A123459</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TANUAPPSEP12</t>
   </si>
   <si>
     <t xml:space="preserve">Acquirer Code</t>
@@ -628,16 +634,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -766,7 +772,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.92"/>
@@ -801,22 +807,22 @@
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="3" t="n">
+        <v>7776668889</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>8758787876</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="3" t="n">
+        <v>7776668889</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -824,323 +830,248 @@
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>8758787877</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="C3" s="3" t="n">
+        <v>7776668890</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>7776668890</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>8758787878</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="C4" s="3" t="n">
+        <v>7776668891</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>7776668891</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>8758787879</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="C5" s="3" t="n">
+        <v>7776668892</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>7776668892</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>8758787870</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>8758787870</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="C6" s="3" t="n">
+        <v>7776668893</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>7776668893</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>9647295710</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>9647295710</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="1" t="s">
+      <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>9049574840</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9049574840</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>8237594032</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>8237594032</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="1" t="s">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>7467464745</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>7467464745</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>9028471826</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>9028471826</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="1" t="s">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>7467464746</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>7467464746</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>7467464747</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>7467464747</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>9049549086</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>7483629150</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>7483629150</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="1" t="s">
+      <c r="E11" s="3" t="n">
+        <v>9049549086</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>6738294739</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>6738294739</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>6029485739</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>6029485739</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>8596837205</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>8596837205</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>6758302759</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>6758302759</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>7869503895</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>7869503895</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>5697869503</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>5697869503</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7"/>
@@ -1207,7 +1138,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="16.47265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.36"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.45"/>
@@ -1227,552 +1158,552 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="P1" s="5" t="s">
         <v>43</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P2" s="5" t="s">
         <v>52</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E3" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="M3" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" s="10" t="s">
+      <c r="P3" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="K3" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="L3" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="M3" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L4" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N4" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="M4" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N4" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>52</v>
+      <c r="O4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N5" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="M5" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N5" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>52</v>
+      <c r="O5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E6" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="L6" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N6" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>52</v>
+      <c r="P6" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="F7" s="4" t="s">
         <v>65</v>
       </c>
+      <c r="F7" s="5" t="s">
+        <v>67</v>
+      </c>
       <c r="G7" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L7" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N7" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="M7" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N7" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>52</v>
+      <c r="O7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H8" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>46</v>
-      </c>
       <c r="J8" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>52</v>
+        <v>71</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="L9" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="M9" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N9" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>52</v>
+      <c r="P9" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>70</v>
+      <c r="A10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="5" t="s">
+      <c r="D10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="O10" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="K10" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="N10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="O10" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="P10" s="5" t="s">
-        <v>52</v>
+      <c r="P10" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="14"/>
       <c r="R11" s="14"/>
@@ -1820,7 +1751,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="16.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.59"/>
   </cols>
@@ -1830,229 +1761,229 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B2" s="10" t="n">
         <v>8</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D2" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F2" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F3" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B4" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D10" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>10786</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -2072,7 +2003,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="16.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.44"/>
@@ -2090,63 +2021,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="N1" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="O1" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="P1" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>120000000008131</v>
@@ -2158,83 +2089,83 @@
         <v>120000000008131</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I2" s="10" t="n">
         <v>5</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="M2" s="10"/>
       <c r="N2" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O2" s="10"/>
       <c r="P2" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="Q2" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H3" s="10"/>
       <c r="I3" s="10" t="n">
         <v>2</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="Q3" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2260,7 +2191,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="15.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.74"/>
@@ -2268,74 +2199,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>133</v>
+      <c r="A8" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2418,7 +2349,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="15.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.5234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.87"/>
@@ -2427,7 +2358,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2441,58 +2372,58 @@
     </row>
     <row r="2" customFormat="false" ht="11.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C2" s="17" t="n">
         <v>7207207201</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C3" s="17" t="n">
         <v>7207207202</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C4" s="17" t="n">
         <v>7207207203</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>7207207205</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2512,7 +2443,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="14" width="17.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="14" width="18.89"/>
@@ -2520,7 +2451,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -2534,21 +2465,21 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>7383838389</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>8</v>
@@ -2557,7 +2488,7 @@
         <v>9886592527</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2577,7 +2508,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.63"/>
@@ -2588,36 +2519,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>7771111110</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>7674527291947120</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
HDFC_MINTOAK BQRV4 Test Cases
</commit_message>
<xml_diff>
--- a/DataProvider/merchant_user_creation.xlsx
+++ b/DataProvider/merchant_user_creation.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="156">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -365,13 +365,13 @@
     <t xml:space="preserve">CYBERSOURCE</t>
   </si>
   <si>
+    <t xml:space="preserve">hdfc_89052195</t>
+  </si>
+  <si>
     <t xml:space="preserve">DV+y0pRK1jhkpBipZ+YtM06XqQGOi1SDwsmOY/K4wqo=</t>
   </si>
   <si>
     <t xml:space="preserve">8bf3bb8f-eb7c-45d2-b227-bf779907d017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ezetap_2020</t>
   </si>
   <si>
     <t xml:space="preserve">SHA1</t>
@@ -766,7 +766,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.92"/>
@@ -1193,7 +1193,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
@@ -1207,7 +1207,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA53"/>
-  <sheetFormatPr defaultColWidth="16.47265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.5" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.36"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.45"/>
@@ -1795,18 +1795,18 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K10" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K10" type="list">
       <formula1>AcquisitionDetails!$AA$52:$AA$52</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I10" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I10" type="list">
       <formula1>AcquisitionDetails!$AA$52:$AA$53</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
@@ -1820,7 +1820,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="16.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.21875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.59"/>
   </cols>
@@ -2058,7 +2058,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
@@ -2072,7 +2072,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="16.19921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.21875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.44"/>
@@ -2148,24 +2148,22 @@
       <c r="B2" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C2" s="10" t="n">
-        <v>120000000008131</v>
-      </c>
-      <c r="D2" s="10" t="n">
-        <v>120000000008131</v>
-      </c>
-      <c r="E2" s="10" t="n">
-        <v>120000000008131</v>
+      <c r="C2" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="H2" s="10" t="s">
         <v>114</v>
       </c>
+      <c r="H2" s="10"/>
       <c r="I2" s="10" t="n">
         <v>5</v>
       </c>
@@ -2239,14 +2237,14 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="Q2:Q3" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="Q2:Q3" type="list">
       <formula1>AcquisitionDetails!$AA$52:$AA$53</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
@@ -2260,7 +2258,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="15.88671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.90234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.74"/>
@@ -2404,7 +2402,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
@@ -2418,7 +2416,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="15.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.5078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.87"/>
@@ -2498,7 +2496,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 Page &amp;P</oddFooter>
@@ -2512,7 +2510,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="13.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.01171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="14" width="17.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="14" width="18.89"/>
@@ -2563,7 +2561,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
@@ -2577,7 +2575,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.63"/>
@@ -2639,7 +2637,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>